<commit_message>
feat: actualizar analitica y sincronizar datos de planilla
</commit_message>
<xml_diff>
--- a/public/PLANILLA GASTOS COMUNES.xlsx
+++ b/public/PLANILLA GASTOS COMUNES.xlsx
@@ -37034,7 +37034,7 @@
         <v>RUTH DAYANA ESTEFANIA BULETRAU REYES</v>
       </c>
       <c r="B490" t="str">
-        <v>7.709.555-1</v>
+        <v>25.544.397-6</v>
       </c>
       <c r="C490" t="str">
         <v/>
@@ -37055,7 +37055,7 @@
         <v>Pendiente</v>
       </c>
       <c r="I490" t="str">
-        <v>2026-04-11T23:32:29.146Z</v>
+        <v>2026-04-11T23:47:14.856Z</v>
       </c>
       <c r="J490">
         <v>958196463</v>

</xml_diff>